<commit_message>
Finalize validated datasets and freshness
</commit_message>
<xml_diff>
--- a/data/exports/entity_mapping_log.xlsx
+++ b/data/exports/entity_mapping_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -748,12 +748,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TechCrunch</t>
+          <t>Google Research</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://techcrunch.com/2026/09/03/qualcomm-backs-ultrahuman-in-70m-round-on-bet-to-turn-smart-rings-into-computers/</t>
+          <t>https://research.google/blog/transfer-learning-for-genomic-prediction-in-underrepresented-populations/</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -762,33 +762,6 @@
         </is>
       </c>
       <c r="E13" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>NEWS</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Google Research</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>https://research.google/blog/transfer-learning-for-genomic-prediction-in-underrepresented-populations/</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
         <is>
           <t>nan</t>
         </is>

</xml_diff>